<commit_message>
Keep archival market labels inactive in canonical Excel export
</commit_message>
<xml_diff>
--- a/exports/fantasy-2026-current.xlsx
+++ b/exports/fantasy-2026-current.xlsx
@@ -164,7 +164,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -234,7 +234,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -304,7 +304,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -374,7 +374,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -444,7 +444,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -724,7 +724,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -1774,7 +1774,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -1984,7 +1984,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2334,7 +2334,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -2404,7 +2404,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -2824,7 +2824,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -2964,7 +2964,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -3174,7 +3174,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -3244,7 +3244,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -3314,7 +3314,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -3454,7 +3454,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -3734,7 +3734,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -3804,7 +3804,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -3944,7 +3944,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -4084,7 +4084,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -4294,7 +4294,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
@@ -4364,7 +4364,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -4574,7 +4574,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -4714,7 +4714,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -4854,7 +4854,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -4924,7 +4924,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -5064,7 +5064,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -5204,7 +5204,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -5274,7 +5274,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -5344,7 +5344,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -5834,7 +5834,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
@@ -6044,7 +6044,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -6114,7 +6114,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
@@ -6184,7 +6184,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
@@ -6254,7 +6254,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
@@ -6324,7 +6324,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
@@ -6394,7 +6394,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
@@ -6464,7 +6464,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
@@ -6534,7 +6534,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
@@ -6604,7 +6604,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr">
@@ -6814,7 +6814,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
@@ -6884,7 +6884,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
@@ -6954,7 +6954,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q99" t="inlineStr">
@@ -7024,7 +7024,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -7094,7 +7094,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -7164,7 +7164,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -7234,7 +7234,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -7304,7 +7304,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -7374,7 +7374,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -7444,7 +7444,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -7514,7 +7514,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -7584,7 +7584,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
@@ -7654,7 +7654,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
@@ -7724,7 +7724,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
@@ -7794,7 +7794,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
@@ -7864,7 +7864,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
@@ -8004,7 +8004,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
@@ -8214,7 +8214,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q117" t="inlineStr">
@@ -8284,7 +8284,7 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr">
@@ -8354,7 +8354,7 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
@@ -8424,7 +8424,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -8494,7 +8494,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -8564,7 +8564,7 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr">
@@ -8634,7 +8634,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr">
@@ -8774,7 +8774,7 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
@@ -8844,7 +8844,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
@@ -8984,7 +8984,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -9124,7 +9124,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
@@ -9334,7 +9334,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
@@ -9404,7 +9404,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -9544,7 +9544,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -9684,7 +9684,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -9754,7 +9754,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -9894,7 +9894,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -9964,7 +9964,7 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -10034,7 +10034,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q144" t="inlineStr">
@@ -10174,7 +10174,7 @@
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q145" t="inlineStr">
@@ -10244,7 +10244,7 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr">
@@ -10314,7 +10314,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q147" t="inlineStr">
@@ -10384,7 +10384,7 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q148" t="inlineStr">
@@ -10454,7 +10454,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q149" t="inlineStr">
@@ -10524,7 +10524,7 @@
       </c>
       <c r="P150" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q150" t="inlineStr">
@@ -10594,7 +10594,7 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q151" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
@@ -10734,7 +10734,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q153" t="inlineStr">
@@ -10804,7 +10804,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q154" t="inlineStr">
@@ -10874,7 +10874,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q155" t="inlineStr">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q156" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q157" t="inlineStr">
@@ -11084,7 +11084,7 @@
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q158" t="inlineStr">
@@ -11154,7 +11154,7 @@
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q159" t="inlineStr">
@@ -11224,7 +11224,7 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q160" t="inlineStr">
@@ -11294,7 +11294,7 @@
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
@@ -11364,7 +11364,7 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q162" t="inlineStr">
@@ -11434,7 +11434,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q163" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr">
@@ -11574,7 +11574,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr">
@@ -11644,7 +11644,7 @@
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr">
@@ -11714,7 +11714,7 @@
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q167" t="inlineStr">
@@ -11784,7 +11784,7 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN_SEASON</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q168" t="inlineStr">
@@ -11959,7 +11959,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -12029,7 +12029,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -12099,7 +12099,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -12169,7 +12169,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -12239,7 +12239,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -12379,7 +12379,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -12449,7 +12449,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -12519,7 +12519,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -12729,7 +12729,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -12799,7 +12799,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -12869,7 +12869,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -12939,7 +12939,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -13009,7 +13009,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -13079,7 +13079,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -13149,7 +13149,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -13219,7 +13219,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -13289,7 +13289,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -13359,7 +13359,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -13499,7 +13499,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
@@ -13569,7 +13569,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
@@ -13639,7 +13639,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -13709,7 +13709,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -13779,7 +13779,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -13849,7 +13849,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -13919,7 +13919,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -14059,7 +14059,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -14129,7 +14129,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -14269,7 +14269,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -14339,7 +14339,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -14409,7 +14409,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -14479,7 +14479,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -14619,7 +14619,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -14689,7 +14689,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -14759,7 +14759,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -14899,7 +14899,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -14969,7 +14969,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -15039,7 +15039,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
@@ -15109,7 +15109,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
@@ -15179,7 +15179,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -15249,7 +15249,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
@@ -15319,7 +15319,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -15389,7 +15389,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -15459,7 +15459,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -15529,7 +15529,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -15599,7 +15599,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -15669,7 +15669,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -15739,7 +15739,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -15809,7 +15809,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr">
@@ -15879,7 +15879,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -15949,7 +15949,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -16019,7 +16019,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -16089,7 +16089,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -16229,7 +16229,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -16299,7 +16299,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -16369,7 +16369,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -16439,7 +16439,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -16509,7 +16509,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -16579,7 +16579,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -16649,7 +16649,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -16719,7 +16719,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -16789,7 +16789,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -16859,7 +16859,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
@@ -16929,7 +16929,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -16999,7 +16999,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -17069,7 +17069,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -17139,7 +17139,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -17209,7 +17209,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -17279,7 +17279,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -17349,7 +17349,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -17419,7 +17419,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -17489,7 +17489,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -17559,7 +17559,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -17629,7 +17629,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -17699,7 +17699,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr">
@@ -17769,7 +17769,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr">
@@ -17839,7 +17839,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -17909,7 +17909,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
@@ -17979,7 +17979,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
@@ -18049,7 +18049,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
@@ -18119,7 +18119,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
@@ -18189,7 +18189,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
@@ -18259,7 +18259,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
@@ -18329,7 +18329,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
@@ -18399,7 +18399,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
@@ -18469,7 +18469,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -18539,7 +18539,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr">
@@ -18609,7 +18609,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
@@ -18679,7 +18679,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
@@ -18749,7 +18749,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q99" t="inlineStr">
@@ -18819,7 +18819,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -18889,7 +18889,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -18959,7 +18959,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -19029,7 +19029,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -19099,7 +19099,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -19169,7 +19169,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -19239,7 +19239,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -19309,7 +19309,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr">
@@ -19379,7 +19379,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr">
@@ -19449,7 +19449,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
@@ -19519,7 +19519,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
@@ -19589,7 +19589,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
@@ -19659,7 +19659,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
@@ -19729,7 +19729,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
@@ -19799,7 +19799,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -19869,7 +19869,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
@@ -19939,7 +19939,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
@@ -20009,7 +20009,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q117" t="inlineStr">
@@ -20079,7 +20079,7 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr">
@@ -20149,7 +20149,7 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
@@ -20219,7 +20219,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -20289,7 +20289,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -20359,7 +20359,7 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr">
@@ -20429,7 +20429,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
@@ -20499,7 +20499,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr">
@@ -20569,7 +20569,7 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
@@ -20639,7 +20639,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
@@ -20709,7 +20709,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
@@ -20779,7 +20779,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
@@ -20849,7 +20849,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -20919,7 +20919,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
@@ -20989,7 +20989,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
@@ -21059,7 +21059,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
@@ -21129,7 +21129,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
@@ -21199,7 +21199,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -21269,7 +21269,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -21339,7 +21339,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -21409,7 +21409,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr">
@@ -21479,7 +21479,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr">
@@ -21549,7 +21549,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -21619,7 +21619,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -21689,7 +21689,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr">
@@ -21759,7 +21759,7 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr">
@@ -21829,7 +21829,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr">
@@ -21899,7 +21899,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q144" t="inlineStr">
@@ -21969,7 +21969,7 @@
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q145" t="inlineStr">
@@ -22039,7 +22039,7 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr">
@@ -22109,7 +22109,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q147" t="inlineStr">
@@ -22179,7 +22179,7 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q148" t="inlineStr">
@@ -22249,7 +22249,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q149" t="inlineStr">
@@ -22319,7 +22319,7 @@
       </c>
       <c r="P150" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q150" t="inlineStr">
@@ -22389,7 +22389,7 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q151" t="inlineStr">
@@ -22459,7 +22459,7 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr">
@@ -22529,7 +22529,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t xml:space="preserve">REACH</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q153" t="inlineStr">
@@ -22599,7 +22599,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q154" t="inlineStr">
@@ -22669,7 +22669,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q155" t="inlineStr">
@@ -22739,7 +22739,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q156" t="inlineStr">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q157" t="inlineStr">
@@ -22879,7 +22879,7 @@
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q158" t="inlineStr">
@@ -22949,7 +22949,7 @@
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q159" t="inlineStr">
@@ -23019,7 +23019,7 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q160" t="inlineStr">
@@ -23089,7 +23089,7 @@
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
@@ -23159,7 +23159,7 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q162" t="inlineStr">
@@ -23229,7 +23229,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q163" t="inlineStr">
@@ -23299,7 +23299,7 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr">
@@ -23369,7 +23369,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t xml:space="preserve">BUY</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr">
@@ -23439,7 +23439,7 @@
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAIR</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr">
@@ -23509,7 +23509,7 @@
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t xml:space="preserve">FADE</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q167" t="inlineStr">
@@ -23579,7 +23579,7 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t xml:space="preserve">IN_SEASON</t>
+          <t xml:space="preserve">MODEL REVIEW</t>
         </is>
       </c>
       <c r="Q168" t="inlineStr">

</xml_diff>

<commit_message>
Refresh canonical Excel after merged player news updates
</commit_message>
<xml_diff>
--- a/exports/fantasy-2026-current.xlsx
+++ b/exports/fantasy-2026-current.xlsx
@@ -4579,7 +4579,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t xml:space="preserve">cam bynum boasts an impressive track record in international games heading into sunday s matchup with the commanders at london s tottenham hotspur stadium the colts safety has made three previous international appearances two in london with the vikings and another in germany last year for indianapolis and has come away 3 0 with 17 tackles two passes defensed an interception and a forced fumble what has contributed to such a boost overseas for the 28 year old he believes a lot of it boils down to the atmosphere whenever i m having fun and feeling loose that s when i play the best football bynum told mike yam on thursday s episode of the nfl report so when i m overseas playing in front of diff</t>
+          <t xml:space="preserve">Will Marcus Mariota lead Washington to a second straight win in relief of Jayden Daniels? | cam bynum boasts an impressive track record in international games heading into sunday s matchup with the commanders at london s tottenham hotspur stadium the colts safety has made three previous international appearances two in london with the vikings and another in germany last year for indianapolis and has come away 3 0 with 17 tackles two passes defensed an interception and a forced fumble what has contributed to such a boost overseas for the 28 year old he believes a lot of it boils down to the atmosphere whenever i m having fun and feeling loose that s when i play the best football bynum told mi</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -7239,7 +7239,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t xml:space="preserve">first round quarterback who even the stingiest draft graders pegged as a day 2 selection teams use fifth rounders and later as qb dart throws all the time the giants lack of 2027 picks is of concern but they can deal with that later with jaxson dart out for the regular season after knee surgery the giants needed to make some sort of move jameis winston has shown he can hold the fort for a spell but it s a serious question if harbaugh will give the boom or bust passer enough | j j mccarthy is ready for a fresh start 34 i didn 39 t anticipate it 34 the 23 year old quarterback said friday four days after the new york giants acquired him from the minnesota vikings for a 2027 fifth round pick 34 </t>
+          <t xml:space="preserve">first round quarterback who even the stingiest draft graders pegged as a day 2 selection teams use fifth rounders and later as qb dart throws all the time the giants lack of 2027 picks is of concern but they can deal with that later with jaxson dart out for the regular season after knee surgery the giants needed to make some sort of move jameis winston has shown he can hold the fort for a spell but it s a serious question if harbaugh will give the boom or bust passer enough | Transaction: Placed QB Jaxson Dart on injured reserve. | Placed QB Jaxson Dart on injured reserve. | transaction placed qb jaxson dart on injured reserve placed qb jaxson dart on injured reserve</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -7519,7 +7519,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t xml:space="preserve">the patriots don 39 t have any answers mack hollins who picked up a taunting penalty while his team trailed 28 3 is playing like the team 39 s best wide receiver which is great for hollins but not a great sign for the team romeo doubs isn 39 t playing like a 17 million player kyle williams was blanketed in coverage on what ended up as maye 39 s second interception and the offense remains totally unable to run the ball so if it 39 s going to get better it</t>
+          <t xml:space="preserve">Patriots preach patience when it comes to receiver WR Romeo Doubs' modest start | patriots preach patience when it comes to receiver wr romeo doubs modest start after the patriots signed him to a four year deal in march doubs is searching for his footing in the offense entering week 4</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -16514,7 +16514,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t xml:space="preserve">cam bynum boasts an impressive track record in international games heading into sunday s matchup with the commanders at london s tottenham hotspur stadium the colts safety has made three previous international appearances two in london with the vikings and another in germany last year for indianapolis and has come away 3 0 with 17 tackles two passes defensed an interception and a forced fumble what has contributed to such a boost overseas for the 28 year old he believes a lot of it boils down to the atmosphere whenever i m having fun and feeling loose that s when i play the best football bynum told mike yam on thursday s episode of the nfl report so when i m overseas playing in front of diff</t>
+          <t xml:space="preserve">Will Marcus Mariota lead Washington to a second straight win in relief of Jayden Daniels? | cam bynum boasts an impressive track record in international games heading into sunday s matchup with the commanders at london s tottenham hotspur stadium the colts safety has made three previous international appearances two in london with the vikings and another in germany last year for indianapolis and has come away 3 0 with 17 tackles two passes defensed an interception and a forced fumble what has contributed to such a boost overseas for the 28 year old he believes a lot of it boils down to the atmosphere whenever i m having fun and feeling loose that s when i play the best football bynum told mi</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -19734,7 +19734,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t xml:space="preserve">the patriots don 39 t have any answers mack hollins who picked up a taunting penalty while his team trailed 28 3 is playing like the team 39 s best wide receiver which is great for hollins but not a great sign for the team romeo doubs isn 39 t playing like a 17 million player kyle williams was blanketed in coverage on what ended up as maye 39 s second interception and the offense remains totally unable to run the ball so if it 39 s going to get better it</t>
+          <t xml:space="preserve">Patriots preach patience when it comes to receiver WR Romeo Doubs' modest start | patriots preach patience when it comes to receiver wr romeo doubs modest start after the patriots signed him to a four year deal in march doubs is searching for his footing in the offense entering week 4</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -20364,7 +20364,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t xml:space="preserve">first round quarterback who even the stingiest draft graders pegged as a day 2 selection teams use fifth rounders and later as qb dart throws all the time the giants lack of 2027 picks is of concern but they can deal with that later with jaxson dart out for the regular season after knee surgery the giants needed to make some sort of move jameis winston has shown he can hold the fort for a spell but it s a serious question if harbaugh will give the boom or bust passer enough | j j mccarthy is ready for a fresh start 34 i didn 39 t anticipate it 34 the 23 year old quarterback said friday four days after the new york giants acquired him from the minnesota vikings for a 2027 fifth round pick 34 </t>
+          <t xml:space="preserve">first round quarterback who even the stingiest draft graders pegged as a day 2 selection teams use fifth rounders and later as qb dart throws all the time the giants lack of 2027 picks is of concern but they can deal with that later with jaxson dart out for the regular season after knee surgery the giants needed to make some sort of move jameis winston has shown he can hold the fort for a spell but it s a serious question if harbaugh will give the boom or bust passer enough | Transaction: Placed QB Jaxson Dart on injured reserve. | Placed QB Jaxson Dart on injured reserve. | transaction placed qb jaxson dart on injured reserve placed qb jaxson dart on injured reserve</t>
         </is>
       </c>
       <c r="R122" t="inlineStr">

</xml_diff>

<commit_message>
Include Word profiles and rank-change records in player admissions
</commit_message>
<xml_diff>
--- a/exports/fantasy-2026-current.xlsx
+++ b/exports/fantasy-2026-current.xlsx
@@ -309,7 +309,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles as he deals with back soreness while wide receiver puka nacua will return from a hip injury after missing the past two games | n count if there were offseason trophies to hand out los angeles would likely be first in line still for as loaded as this roster is it s imperative the rams stiff arm distractions and keep th</t>
+          <t xml:space="preserve">Sources: Rams don't intend to limit Puka Nacua's workload | The Rams do not intend to limit Puka Nacua's workload Sunday against the Eagles, sources told ESPN. | sources rams don t intend to limit puka nacua s workload the rams do not intend to limit puka nacua s workload sunday against the eagles sources told espn | Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles </t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Can Terry McLaurin overcome a tough Eagles defense? | nfl fantasy 2026 start x27 em sit x27 em wide receivers for week 1 which jaguars receiver is primed to star in the opener can terry mclaurin overcome a tough eagles defense check out all of matt okada x27 s fantasy wr starts and sits for week 1 of the 2026 nfl season</t>
+          <t xml:space="preserve">Commanders WR Terry McLaurin inactive after Friday injury | Commanders wide receiver Terry McLaurin will not play against the Colts because of a hamstring injury suffered in practice Friday. | commanders wr terry mclaurin inactive after friday injury commanders wide receiver terry mclaurin will not play against the colts because of a hamstring injury suffered in practice friday</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t xml:space="preserve">en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of camp tight end sam laporta is the name to watch on offense but the defense has greater concerns brian branch suffered a late season achilles tear and while the lions haven t put a hard timeline on the safety s recovery it will be a surprise if he s good to go to ope</t>
+          <t xml:space="preserve">Sources: Sam LaPorta, Lions break off contract talks | The Lions and star tight end Sam LaPorta have broken off contract talks, sources told NFL Network, after attempting to work out a long-term deal for the first few weeks of the season. | sources sam laporta lions break off contract talks the lions and star tight end sam laporta have broken off contract talks sources told nfl network after attempting to work out a long term deal for the first few weeks of the season | en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of </t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Synchronized to Washington across team, Overall, Regression, Environment and Step 7; old unsigned/landing-spot wording removed.</t>
+          <t xml:space="preserve">com nfl player id 4361577 dyami brown dyami brown a and a href https www espn com nfl player id 4567156 treylon burks trey burks a can fill mclaurin s x receiver role as can a href https www espn com nfl player id 2976212 stefon diggs stefon diggs a who has started at the flanker position opposite mclaurin diggs leads washington with 13 receptions and three touchdown catches while mclaurin has a team best 141 receiving yards p p washington does return tight end a href https www espn com nfl</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Carolina Panthers are monitoring starting wide receiver Jalen Coker's quadriceps injury ahead of their Week 4 "Sunday Night Football" matchup with the Detroit Lions. | panthers in wait and see mode with leading receiver coker quad the carolina panthers are monitoring starting wide receiver jalen coker s quadriceps injury ahead of their week 4 sunday night football matchup with the detroit lions</t>
+          <t xml:space="preserve">Wide receiver Jalen Coker is also unlikely to play against the Lions, sources told ESPN. | panthers put legette on ir coker also likely out vs lions the panthers have placed 2024 first round pick xavier legette on injured reserve ahead of sunday s prime time matchup against the lions wide receiver jalen coker is also unlikely to play against the lions sources told espn</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -9479,7 +9479,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t xml:space="preserve">see him go through the workouts the commanders leave for london on tuesday evening and are scheduled to practice wednesday through friday before hosting the colts at tottenham hotspur stadium on sunday at 9 30 a m et linebacker frankie luvu groin and tight end chig okonkwo hamstring will also return to practice in some form this week after missing the last two games because of injury the status of right guard sam cosmi concussion and safety nick cross internal injury however will be decided later after each player undergoes further testing</t>
+          <t xml:space="preserve">who has started at the flanker position opposite mclaurin diggs leads washington with 13 receptions and three touchdown catches while mclaurin has a team best 141 receiving yards p p washington does return tight end a href https www espn com nfl player id 4360635 chig okonkwo chig okonkwo a who missed the past two games with a hamstring injury p</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buccaneers QB Baker Mayfield out at least 3 weeks with thumb injury; | Jalon Daniels will start at quarterback for the Buccaneers with Baker Mayfield sidelined by his thumb injury. | for the first time in four years the buccaneers will be starting someone other than baker mayfield at quarterback in week 4 bucs head coach todd bowles told reporters on monday that mayfield will miss a minimum of three weeks after dislocating his right thumb in the team s 23 16 loss to the vikings on sunday tampa bay will start undrafted rookie jalon daniels in mayfield s place when it hosts the 1 2 packers on oct 4 daniels went 0 for 3 passing with a game ending interception after coming on in relief of mayfie</t>
+          <t xml:space="preserve">Sources: Baker Mayfield return hinges on when QB can grip football | Baker Mayfield is expected to miss anywhere from three to six weeks, sources told ESPN, depending on how quickly the Bucs QB can grip the football. | p a data clubhouse guid 13e8b157 a75a ff24 ae91 fa3d52ddf204 href https www espn com nfl team name tb tampa bay buccaneers tampa bay buccaneers a head coach todd bowles says a data player guid 5bb4376a d089 e3e4 e49a 44f1d709a012 href https www espn com nfl player id 3052587 baker mayfield baker mayfield a will miss at least three weeks due to his dislocated right thumb but that is the minimum p p there is a flipside scenario as well p p sources told espn that mayfield is deal</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12174,7 +12174,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles as he deals with back soreness while wide receiver puka nacua will return from a hip injury after missing the past two games | n count if there were offseason trophies to hand out los angeles would likely be first in line still for as loaded as this roster is it s imperative the rams stiff arm distractions and keep th</t>
+          <t xml:space="preserve">Sources: Rams don't intend to limit Puka Nacua's workload | The Rams do not intend to limit Puka Nacua's workload Sunday against the Eagles, sources told ESPN. | sources rams don t intend to limit puka nacua s workload the rams do not intend to limit puka nacua s workload sunday against the eagles sources told espn | Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles </t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -15394,7 +15394,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Can Terry McLaurin overcome a tough Eagles defense? | nfl fantasy 2026 start x27 em sit x27 em wide receivers for week 1 which jaguars receiver is primed to star in the opener can terry mclaurin overcome a tough eagles defense check out all of matt okada x27 s fantasy wr starts and sits for week 1 of the 2026 nfl season</t>
+          <t xml:space="preserve">Commanders WR Terry McLaurin inactive after Friday injury | Commanders wide receiver Terry McLaurin will not play against the Colts because of a hamstring injury suffered in practice Friday. | commanders wr terry mclaurin inactive after friday injury commanders wide receiver terry mclaurin will not play against the colts because of a hamstring injury suffered in practice friday</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -16304,7 +16304,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t xml:space="preserve">en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of camp tight end sam laporta is the name to watch on offense but the defense has greater concerns brian branch suffered a late season achilles tear and while the lions haven t put a hard timeline on the safety s recovery it will be a surprise if he s good to go to ope</t>
+          <t xml:space="preserve">Sources: Sam LaPorta, Lions break off contract talks | The Lions and star tight end Sam LaPorta have broken off contract talks, sources told NFL Network, after attempting to work out a long-term deal for the first few weeks of the season. | sources sam laporta lions break off contract talks the lions and star tight end sam laporta have broken off contract talks sources told nfl network after attempting to work out a long term deal for the first few weeks of the season | en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of </t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -19874,7 +19874,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Carolina Panthers are monitoring starting wide receiver Jalen Coker's quadriceps injury ahead of their Week 4 "Sunday Night Football" matchup with the Detroit Lions. | panthers in wait and see mode with leading receiver coker quad the carolina panthers are monitoring starting wide receiver jalen coker s quadriceps injury ahead of their week 4 sunday night football matchup with the detroit lions</t>
+          <t xml:space="preserve">Wide receiver Jalen Coker is also unlikely to play against the Lions, sources told ESPN. | panthers put legette on ir coker also likely out vs lions the panthers have placed 2024 first round pick xavier legette on injured reserve ahead of sunday s prime time matchup against the lions wide receiver jalen coker is also unlikely to play against the lions sources told espn</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -19944,7 +19944,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t xml:space="preserve">see him go through the workouts the commanders leave for london on tuesday evening and are scheduled to practice wednesday through friday before hosting the colts at tottenham hotspur stadium on sunday at 9 30 a m et linebacker frankie luvu groin and tight end chig okonkwo hamstring will also return to practice in some form this week after missing the last two games because of injury the status of right guard sam cosmi concussion and safety nick cross internal injury however will be decided later after each player undergoes further testing</t>
+          <t xml:space="preserve">who has started at the flanker position opposite mclaurin diggs leads washington with 13 receptions and three touchdown catches while mclaurin has a team best 141 receiving yards p p washington does return tight end a href https www espn com nfl player id 4360635 chig okonkwo chig okonkwo a who missed the past two games with a hamstring injury p</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -20434,7 +20434,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Synchronized to Washington across team, Overall, Regression, Environment and Step 7; old unsigned/landing-spot wording removed.</t>
+          <t xml:space="preserve">com nfl player id 4361577 dyami brown dyami brown a and a href https www espn com nfl player id 4567156 treylon burks trey burks a can fill mclaurin s x receiver role as can a href https www espn com nfl player id 2976212 stefon diggs stefon diggs a who has started at the flanker position opposite mclaurin diggs leads washington with 13 receptions and three touchdown catches while mclaurin has a team best 141 receiving yards p p washington does return tight end a href https www espn com nfl</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -22814,7 +22814,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buccaneers QB Baker Mayfield out at least 3 weeks with thumb injury; | Jalon Daniels will start at quarterback for the Buccaneers with Baker Mayfield sidelined by his thumb injury. | for the first time in four years the buccaneers will be starting someone other than baker mayfield at quarterback in week 4 bucs head coach todd bowles told reporters on monday that mayfield will miss a minimum of three weeks after dislocating his right thumb in the team s 23 16 loss to the vikings on sunday tampa bay will start undrafted rookie jalon daniels in mayfield s place when it hosts the 1 2 packers on oct 4 daniels went 0 for 3 passing with a game ending interception after coming on in relief of mayfie</t>
+          <t xml:space="preserve">Sources: Baker Mayfield return hinges on when QB can grip football | Baker Mayfield is expected to miss anywhere from three to six weeks, sources told ESPN, depending on how quickly the Bucs QB can grip the football. | p a data clubhouse guid 13e8b157 a75a ff24 ae91 fa3d52ddf204 href https www espn com nfl team name tb tampa bay buccaneers tampa bay buccaneers a head coach todd bowles says a data player guid 5bb4376a d089 e3e4 e49a 44f1d709a012 href https www espn com nfl player id 3052587 baker mayfield baker mayfield a will miss at least three weeks due to his dislocated right thumb but that is the minimum p p there is a flipside scenario as well p p sources told espn that mayfield is deal</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">

</xml_diff>

<commit_message>
Synchronize base admission Excel with current canonical player news
</commit_message>
<xml_diff>
--- a/exports/fantasy-2026-current.xlsx
+++ b/exports/fantasy-2026-current.xlsx
@@ -309,7 +309,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles as he deals with back soreness while wide receiver puka nacua will return from a hip injury after missing the past two games | n count if there were offseason trophies to hand out los angeles would likely be first in line still for as loaded as this roster is it s imperative the rams stiff arm distractions and keep th</t>
+          <t xml:space="preserve">Sources: Rams don't intend to limit Puka Nacua's workload | The Rams do not intend to limit Puka Nacua's workload Sunday against the Eagles, sources told ESPN. | sources rams don t intend to limit puka nacua s workload the rams do not intend to limit puka nacua s workload sunday against the eagles sources told espn | Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles </t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Can Terry McLaurin overcome a tough Eagles defense? | nfl fantasy 2026 start x27 em sit x27 em wide receivers for week 1 which jaguars receiver is primed to star in the opener can terry mclaurin overcome a tough eagles defense check out all of matt okada x27 s fantasy wr starts and sits for week 1 of the 2026 nfl season</t>
+          <t xml:space="preserve">Commanders WR Terry McLaurin inactive after Friday injury | Commanders wide receiver Terry McLaurin will not play against the Colts because of a hamstring injury suffered in practice Friday. | commanders wr terry mclaurin inactive after friday injury commanders wide receiver terry mclaurin will not play against the colts because of a hamstring injury suffered in practice friday</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t xml:space="preserve">en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of camp tight end sam laporta is the name to watch on offense but the defense has greater concerns brian branch suffered a late season achilles tear and while the lions haven t put a hard timeline on the safety s recovery it will be a surprise if he s good to go to ope</t>
+          <t xml:space="preserve">Sources: Sam LaPorta, Lions break off contract talks | The Lions and star tight end Sam LaPorta have broken off contract talks, sources told NFL Network, after attempting to work out a long-term deal for the first few weeks of the season. | sources sam laporta lions break off contract talks the lions and star tight end sam laporta have broken off contract talks sources told nfl network after attempting to work out a long term deal for the first few weeks of the season | en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of </t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -6679,7 +6679,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Synchronized to Washington across team, Overall, Regression, Environment and Step 7; old unsigned/landing-spot wording removed.</t>
+          <t xml:space="preserve">com nfl player id 4361577 dyami brown dyami brown a and a href https www espn com nfl player id 4567156 treylon burks trey burks a can fill mclaurin s x receiver role as can a href https www espn com nfl player id 2976212 stefon diggs stefon diggs a who has started at the flanker position opposite mclaurin diggs leads washington with 13 receptions and three touchdown catches while mclaurin has a team best 141 receiving yards p p washington does return tight end a href https www espn com nfl</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -7939,7 +7939,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Carolina Panthers are monitoring starting wide receiver Jalen Coker's quadriceps injury ahead of their Week 4 "Sunday Night Football" matchup with the Detroit Lions. | panthers in wait and see mode with leading receiver coker quad the carolina panthers are monitoring starting wide receiver jalen coker s quadriceps injury ahead of their week 4 sunday night football matchup with the detroit lions</t>
+          <t xml:space="preserve">Wide receiver Jalen Coker is also unlikely to play against the Lions, sources told ESPN. | panthers put legette on ir coker also likely out vs lions the panthers have placed 2024 first round pick xavier legette on injured reserve ahead of sunday s prime time matchup against the lions wide receiver jalen coker is also unlikely to play against the lions sources told espn</t>
         </is>
       </c>
       <c r="R113" t="inlineStr">
@@ -9479,7 +9479,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t xml:space="preserve">see him go through the workouts the commanders leave for london on tuesday evening and are scheduled to practice wednesday through friday before hosting the colts at tottenham hotspur stadium on sunday at 9 30 a m et linebacker frankie luvu groin and tight end chig okonkwo hamstring will also return to practice in some form this week after missing the last two games because of injury the status of right guard sam cosmi concussion and safety nick cross internal injury however will be decided later after each player undergoes further testing</t>
+          <t xml:space="preserve">who has started at the flanker position opposite mclaurin diggs leads washington with 13 receptions and three touchdown catches while mclaurin has a team best 141 receiving yards p p washington does return tight end a href https www espn com nfl player id 4360635 chig okonkwo chig okonkwo a who missed the past two games with a hamstring injury p</t>
         </is>
       </c>
       <c r="R135" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buccaneers QB Baker Mayfield out at least 3 weeks with thumb injury; | Jalon Daniels will start at quarterback for the Buccaneers with Baker Mayfield sidelined by his thumb injury. | for the first time in four years the buccaneers will be starting someone other than baker mayfield at quarterback in week 4 bucs head coach todd bowles told reporters on monday that mayfield will miss a minimum of three weeks after dislocating his right thumb in the team s 23 16 loss to the vikings on sunday tampa bay will start undrafted rookie jalon daniels in mayfield s place when it hosts the 1 2 packers on oct 4 daniels went 0 for 3 passing with a game ending interception after coming on in relief of mayfie</t>
+          <t xml:space="preserve">Sources: Baker Mayfield return hinges on when QB can grip football | Baker Mayfield is expected to miss anywhere from three to six weeks, sources told ESPN, depending on how quickly the Bucs QB can grip the football. | p a data clubhouse guid 13e8b157 a75a ff24 ae91 fa3d52ddf204 href https www espn com nfl team name tb tampa bay buccaneers tampa bay buccaneers a head coach todd bowles says a data player guid 5bb4376a d089 e3e4 e49a 44f1d709a012 href https www espn com nfl player id 3052587 baker mayfield baker mayfield a will miss at least three weeks due to his dislocated right thumb but that is the minimum p p there is a flipside scenario as well p p sources told espn that mayfield is deal</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -12174,7 +12174,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles as he deals with back soreness while wide receiver puka nacua will return from a hip injury after missing the past two games | n count if there were offseason trophies to hand out los angeles would likely be first in line still for as loaded as this roster is it s imperative the rams stiff arm distractions and keep th</t>
+          <t xml:space="preserve">Sources: Rams don't intend to limit Puka Nacua's workload | The Rams do not intend to limit Puka Nacua's workload Sunday against the Eagles, sources told ESPN. | sources rams don t intend to limit puka nacua s workload the rams do not intend to limit puka nacua s workload sunday against the eagles sources told espn | Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles </t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -15394,7 +15394,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Can Terry McLaurin overcome a tough Eagles defense? | nfl fantasy 2026 start x27 em sit x27 em wide receivers for week 1 which jaguars receiver is primed to star in the opener can terry mclaurin overcome a tough eagles defense check out all of matt okada x27 s fantasy wr starts and sits for week 1 of the 2026 nfl season</t>
+          <t xml:space="preserve">Commanders WR Terry McLaurin inactive after Friday injury | Commanders wide receiver Terry McLaurin will not play against the Colts because of a hamstring injury suffered in practice Friday. | commanders wr terry mclaurin inactive after friday injury commanders wide receiver terry mclaurin will not play against the colts because of a hamstring injury suffered in practice friday</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
@@ -16304,7 +16304,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t xml:space="preserve">en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of camp tight end sam laporta is the name to watch on offense but the defense has greater concerns brian branch suffered a late season achilles tear and while the lions haven t put a hard timeline on the safety s recovery it will be a surprise if he s good to go to ope</t>
+          <t xml:space="preserve">Sources: Sam LaPorta, Lions break off contract talks | The Lions and star tight end Sam LaPorta have broken off contract talks, sources told NFL Network, after attempting to work out a long-term deal for the first few weeks of the season. | sources sam laporta lions break off contract talks the lions and star tight end sam laporta have broken off contract talks sources told nfl network after attempting to work out a long term deal for the first few weeks of the season | en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of </t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -19874,7 +19874,7 @@
       </c>
       <c r="Q115" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Carolina Panthers are monitoring starting wide receiver Jalen Coker's quadriceps injury ahead of their Week 4 "Sunday Night Football" matchup with the Detroit Lions. | panthers in wait and see mode with leading receiver coker quad the carolina panthers are monitoring starting wide receiver jalen coker s quadriceps injury ahead of their week 4 sunday night football matchup with the detroit lions</t>
+          <t xml:space="preserve">Wide receiver Jalen Coker is also unlikely to play against the Lions, sources told ESPN. | panthers put legette on ir coker also likely out vs lions the panthers have placed 2024 first round pick xavier legette on injured reserve ahead of sunday s prime time matchup against the lions wide receiver jalen coker is also unlikely to play against the lions sources told espn</t>
         </is>
       </c>
       <c r="R115" t="inlineStr">
@@ -19944,7 +19944,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t xml:space="preserve">see him go through the workouts the commanders leave for london on tuesday evening and are scheduled to practice wednesday through friday before hosting the colts at tottenham hotspur stadium on sunday at 9 30 a m et linebacker frankie luvu groin and tight end chig okonkwo hamstring will also return to practice in some form this week after missing the last two games because of injury the status of right guard sam cosmi concussion and safety nick cross internal injury however will be decided later after each player undergoes further testing</t>
+          <t xml:space="preserve">who has started at the flanker position opposite mclaurin diggs leads washington with 13 receptions and three touchdown catches while mclaurin has a team best 141 receiving yards p p washington does return tight end a href https www espn com nfl player id 4360635 chig okonkwo chig okonkwo a who missed the past two games with a hamstring injury p</t>
         </is>
       </c>
       <c r="R116" t="inlineStr">
@@ -20434,7 +20434,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Synchronized to Washington across team, Overall, Regression, Environment and Step 7; old unsigned/landing-spot wording removed.</t>
+          <t xml:space="preserve">com nfl player id 4361577 dyami brown dyami brown a and a href https www espn com nfl player id 4567156 treylon burks trey burks a can fill mclaurin s x receiver role as can a href https www espn com nfl player id 2976212 stefon diggs stefon diggs a who has started at the flanker position opposite mclaurin diggs leads washington with 13 receptions and three touchdown catches while mclaurin has a team best 141 receiving yards p p washington does return tight end a href https www espn com nfl</t>
         </is>
       </c>
       <c r="R123" t="inlineStr">
@@ -22814,7 +22814,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Buccaneers QB Baker Mayfield out at least 3 weeks with thumb injury; | Jalon Daniels will start at quarterback for the Buccaneers with Baker Mayfield sidelined by his thumb injury. | for the first time in four years the buccaneers will be starting someone other than baker mayfield at quarterback in week 4 bucs head coach todd bowles told reporters on monday that mayfield will miss a minimum of three weeks after dislocating his right thumb in the team s 23 16 loss to the vikings on sunday tampa bay will start undrafted rookie jalon daniels in mayfield s place when it hosts the 1 2 packers on oct 4 daniels went 0 for 3 passing with a game ending interception after coming on in relief of mayfie</t>
+          <t xml:space="preserve">Sources: Baker Mayfield return hinges on when QB can grip football | Baker Mayfield is expected to miss anywhere from three to six weeks, sources told ESPN, depending on how quickly the Bucs QB can grip the football. | p a data clubhouse guid 13e8b157 a75a ff24 ae91 fa3d52ddf204 href https www espn com nfl team name tb tampa bay buccaneers tampa bay buccaneers a head coach todd bowles says a data player guid 5bb4376a d089 e3e4 e49a 44f1d709a012 href https www espn com nfl player id 3052587 baker mayfield baker mayfield a will miss at least three weeks due to his dislocated right thumb but that is the minimum p p there is a flipside scenario as well p p sources told espn that mayfield is deal</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">

</xml_diff>

<commit_message>
Refresh canonical Excel export after main reconciliation
</commit_message>
<xml_diff>
--- a/exports/fantasy-2026-current.xlsx
+++ b/exports/fantasy-2026-current.xlsx
@@ -309,7 +309,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sources: Rams don't intend to limit Puka Nacua's workload | The Rams do not intend to limit Puka Nacua's workload Sunday against the Eagles, sources told ESPN. | sources rams don t intend to limit puka nacua s workload the rams do not intend to limit puka nacua s workload sunday against the eagles sources told espn | Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles </t>
+          <t xml:space="preserve">n count if there were offseason trophies to hand out los angeles would likely be first in line still for as loaded as this roster is it s imperative the rams stiff arm distractions and keep their heads from getting too high into the clouds puka nacua has a looming potentially top of the market extension and he needs to continue working on himself after a stint in rehab l a already caused a stir when it shocked the nfl world by drafting quarterback ty simpson with the 13th overall pick</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -379,7 +379,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Bengals WR Ja'Marr Chase suffers concussion in loss to Jaguars | Bengals wide receiver Ja'Marr Chase has been ruled out against the Jaguars with a concussion.</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t xml:space="preserve">p with 28 seconds left in the fourth quarter sunday afternoon a data clubhouse guid 38248455 3da4 84e4 8090 98b5cc38ffdc href https www espn com nfl team name bal baltimore ravens baltimore ravens a cornerback a data player guid 0fa246a4 1068 3be1 9d79 42844aeedbce href https www espn com nfl player id 4601278 nate wiggins nate wiggins a batted away a pass from a data clubhouse guid b0fc8fb7 9dbe e574 9008 6f0ee7c6b234 href https www espn com nfl team name dal dallas cowboys dallas cowboys a wide receiver a data player guid 2994891b 8927 33cb 6999 e809560d0545 href https www espn com nfl player id 4241389 ceedee lamb ceedee lamb a near the goal line making what many thought was a clutch defe</t>
+          <t xml:space="preserve">CeeDee Lamb's 17 catches, go-ahead score power Cowboys | CeeDee Lamb returned to Houston and caught 17 passes for 189 yards, including the game-winning, 12-yard touchdown with 40 seconds to go, as a large number of family members watched from the stands. | ceedee lamb s 17 catches go ahead score power cowboys ceedee lamb returned to houston and caught 17 passes for 189 yards including the game winning 12 yard touchdown with 40 seconds to go as a large number of family members watched from the stands | Can CeeDee Lamb finish as the overall WR1 in fantasy this season? | can ceedee lamb finish as the overall wr1 in fantasy this season can ceedee lamb finish as the overall wr1 in fantasy this se</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vikings WR Justin Jefferson (ankle) out Sunday against Dolphins | Justin Jefferson (ankle) has been ruled out of the team&amp;#x27;s upcoming game against the Dolphins, head coach Kevin O&amp;#x27;Connell said Friday. | vikings wr justin jefferson ankle out sunday against dolphins the minnesota vikings will be without their two time all pro wide receiver on sunday justin jefferson ankle has been ruled out of the team x27 s upcoming game against the dolphins head coach kevin o x27 connell said friday | Vikings' Justin Jefferson out vs. | Vikings WR Justin Jefferson won't play against the Dolphins because of a sprained left ankle, but coach Kevin O'Connell is hopeful he can return in Week 5 vs. | viki</t>
+          <t xml:space="preserve">Vikings WR Justin Jefferson (ankle) out Sunday against Dolphins | Justin Jefferson (ankle) has been ruled out of the team&amp;#x27;s upcoming game against the Dolphins, head coach Kevin O&amp;#x27;Connell said Friday. | vikings wr justin jefferson ankle out sunday against dolphins the minnesota vikings will be without their two time all pro wide receiver on sunday justin jefferson ankle has been ruled out of the team x27 s upcoming game against the dolphins head coach kevin o x27 connell said friday</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t xml:space="preserve">very big down for us in these first two games and today we were not good enough and i wasn 39 t good enough fourth down i wasn 39 t good enough as well 34 the first half included encouraging signs for the running game saquon barkley returned from last week 39 s stinger and rushed for 73 yards before halftime his second most in the first half since the start of last season but he finished with 82 yards that shows you how the second half went 34 we know the</t>
+          <t xml:space="preserve">Eagles RB Saquon Barkley leaves loss with hamstring injury | Eagles running back Saquon Barkley has been ruled out of Sunday's game against the Rams with a hamstring injury. | eagles rb saquon barkley leaves loss with hamstring injury eagles running back saquon barkley has been ruled out of sunday s game against the rams with a hamstring injury</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who unseats Josh Allen at the top of Nick Shook&amp;#x27;s QB rankings? | nfl and the longest of herbert s career the chargers failed to capitalize on five forced turnovers on sunday as the offense struggled to punch in scores going 1 of 4 in the red zone as the defense gave l a repeated chances to thwart josh allen s bills herbert and co never found a groove after three weeks it s been a rusty operation and herbert doesn t appear comfortable in the scheme yet the interior of the offensive line getting repeatedly blasted doesn t help also the pass catching corps</t>
+          <t xml:space="preserve">is still turning the ball over at a discomforting rate the running game remains an issue the pass rush hasn 39 t been anything special but with their quarterback finally playing like the guy who can carry a team and with their defense slowing down josh allen and the bills like no other unit had everything is on the table for the patriots of course a lot of that is because of maye the disasters of his first three weeks were pretty much gone with allen on the opposing sideline maye certainly</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">— Carolina Panthers coach Dave Canales was a little worried after Bryce Young and Tetairoa McMillan had some issues connecting on passes in practice. | young mcmillan connect for 2 tds to lead panthers past lions 32 26 carolina panthers coach dave canales was a little worried after bryce young and tetairoa mcmillan had some issues connecting on passes in practice</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t xml:space="preserve">jacksonville fla jacksonville jaguars cornerback travis hunter ended up with the football from his first nfl interception hunter spun the ball in celebration and then danced in the end zone after picking off a pass from new england patriots quarterback drake maye late in the second quarter sunday a patriots ball boy picked it up and refused to give it to jaguars veteran defensive end josh hines allen even screaming hey you can t touch me when hines allen tried to grab the ball the ball boy appeared to try to push hines allen away nfl players are allowed to keep game balls although they get charged a hefty price by the league hines allen tried to knock this one out of the ball boy s hands bef</t>
+          <t xml:space="preserve">Drake Maye rebounds as Patriots hand Bills first defeat | Drake Maye snapped out of his early-season slide with a clutch performance as the New England Patriots upset the Buffalo Bills 29-26 at Highmark Stadium in a result that coach Mike Vrabel highlighted as critical for the defending AFC champions. | drake maye rebounds as patriots hand bills first defeat drake maye snapped out of his early season slide with a clutch performance as the new england patriots upset the buffalo bills 29 26 at highmark stadium in a result that coach mike vrabel highlighted as critical for the defending afc champions | Why Adam Rank is still rolling with Drake Maye as a fantasy starter for now | why adam rank i</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t xml:space="preserve">NFL news roundup: Lamar Jackson (back) limited at practice; | nfl news roundup lamar jackson back limited at practice falcons extend dt gervon dexter nfl com keeps you up to date with all of the latest league news from around the nfl visit nfl com x27 s transaction hub for a daily breakdown</t>
+          <t xml:space="preserve">Ravens quarterback Lamar Jackson exits win over Titans early due to ankle injury | Baltimore Ravens quarterback Lamar Jackson suffered an ankle injury in the first half of Sunday&amp;#x27;s 24-18 win over the Tennessee Titans and did not return. | baltimore ravens quarterback lamar jackson suffered an ankle injury in the first half of sunday s 24 18 win over the tennessee titans and did not return jackson appeared to suffer the injury when he was sacked on one of the final plays of the first half lamar s dealing with a little bit of an ankle head coach jesse minter told reporters after the game don t know enough about it right now we ll have to see where that s at nfl network insider ian rapopor</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Michael Florio: Fantasy managers shouldn't think twice about starting Javonte Williams | michael florio fantasy managers shouldn t think twice about starting javonte williams michael florio fantasy managers shouldn t think twice about starting javonte williams</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sources: Sam LaPorta, Lions break off contract talks | The Lions and star tight end Sam LaPorta have broken off contract talks, sources told NFL Network, after attempting to work out a long-term deal for the first few weeks of the season. | sources sam laporta lions break off contract talks the lions and star tight end sam laporta have broken off contract talks sources told nfl network after attempting to work out a long term deal for the first few weeks of the season | en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of </t>
+          <t xml:space="preserve">en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of camp tight end sam laporta is the name to watch on offense but the defense has greater concerns brian branch suffered a late season achilles tear and while the lions haven t put a hard timeline on the safety s recovery it will be a surprise if he s good to go to ope</t>
         </is>
       </c>
       <c r="R58" t="inlineStr">
@@ -4579,7 +4579,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Will Marcus Mariota lead Washington to a second straight win in relief of Jayden Daniels? | cam bynum boasts an impressive track record in international games heading into sunday s matchup with the commanders at london s tottenham hotspur stadium the colts safety has made three previous international appearances two in london with the vikings and another in germany last year for indianapolis and has come away 3 0 with 17 tackles two passes defensed an interception and a forced fumble what has contributed to such a boost overseas for the 28 year old he believes a lot of it boils down to the atmosphere whenever i m having fun and feeling loose that s when i play the best football bynum told mi</t>
+          <t xml:space="preserve">ruled out at halftime mariota was playing in place of washington starter jayden daniels who has been sidelined the last two weeks after dislocating his left elbow on sept 20 commanders coach dan quinn said after the loss that mariota is feared to have aggravated an mcl injury that sidelined him in 2022 the vet qb will undergo testing to confirm the nature of the injury mariota suffered the knee injury on a third down sack midway through the first quarter when indy defensive end laiatu latu landed on the veteran qb s right leg mariota went to the locker room and was replaced by kaliakmanis with washington leading 6 0 this was kaliakmanis first nfl regular season game appearance the 23 year ol</t>
         </is>
       </c>
       <c r="R65" t="inlineStr">
@@ -6329,7 +6329,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t xml:space="preserve">— The Carolina Panthers found themselves in a precarious position last November, facing a red hot Matthew Stafford without three defensive starters, including standout cornerback Jaycee Horn.</t>
+          <t xml:space="preserve">Matthew Stafford says Nacua 'played like Puka' in return for Rams</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -6609,7 +6609,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Placed WR Jayden Reed on injured reserve. | transaction signed g kevin zeitler placed wr jayden reed on injured reserve signed dt david blay and wr coleman owen to the practice squad signed g kevin zeitler placed wr jayden reed on injured reserve signed dt david blay and wr coleman owen to the practice squad | Placed WR Jayden Reed on injured reserve.</t>
+          <t xml:space="preserve">39 s such an impact player on our defense 34 if cooper 39 s injury ends his season it will be the third such hit to green bay 39 s starting lineup this season right tackle zach bako bewele torn patellar tendon and wide receiver jayden reed neck are both out for the year too the packers will now rely on special teams captain and linebacker isaiah mcduffie to fill cooper 39 s spot in the starting lineup alongside veteran zaire franklin lafleur was visibly frustrated during his postgame press conference likely | Placed WR Jayden Reed on injured reserve. | transaction signed g kevin zeitler placed wr jayden reed on injured reserve signed dt david blay and wr coleman owen to the practice squad si</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -7169,7 +7169,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seahawks place RB Jadarian Price (chest) on injured reserve | Running back Jadarian Price&amp;#x27;s slow start to his rookie season just hit another snag. | seahawks place rb jadarian price chest on injured reserve running back jadarian price x27 s slow start to his rookie season just hit another snag the seahawks are placing price on injured reserve due to a chest injury espn x27 s adam schefter reported saturday | Seahawks place RB Jadarian Price (chest) on IR | The Seattle Seahawks are placing starting running back Jadarian Price on injured reserve, the team announced Saturday. | seahawks place rb jadarian price chest on ir the seattle seahawks are placing starting running back jadarian pric</t>
+          <t xml:space="preserve">Seahawks place RB Jadarian Price (chest) on injured reserve | Running back Jadarian Price&amp;#x27;s slow start to his rookie season just hit another snag. | seahawks place rb jadarian price chest on injured reserve running back jadarian price x27 s slow start to his rookie season just hit another snag the seahawks are placing price on injured reserve due to a chest injury espn x27 s adam schefter reported saturday</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -9619,7 +9619,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sources: Baker Mayfield return hinges on when QB can grip football | Baker Mayfield is expected to miss anywhere from three to six weeks, sources told ESPN, depending on how quickly the Bucs QB can grip the football. | p a data clubhouse guid 13e8b157 a75a ff24 ae91 fa3d52ddf204 href https www espn com nfl team name tb tampa bay buccaneers tampa bay buccaneers a head coach todd bowles says a data player guid 5bb4376a d089 e3e4 e49a 44f1d709a012 href https www espn com nfl player id 3052587 baker mayfield baker mayfield a will miss at least three weeks due to his dislocated right thumb but that is the minimum p p there is a flipside scenario as well p p sources told espn that mayfield is deal</t>
+          <t xml:space="preserve">Sources: Baker Mayfield return hinges on when QB can grip football | Baker Mayfield is expected to miss anywhere from three to six weeks, sources told ESPN, depending on how quickly the Buccaneers quarterback can grip the football. | sources baker mayfield return hinges on when qb can grip football baker mayfield is expected to miss anywhere from three to six weeks sources told espn depending on how quickly the buccaneers quarterback can grip the football</t>
         </is>
       </c>
       <c r="R137" t="inlineStr">
@@ -9689,7 +9689,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t xml:space="preserve">an offense playing as if it s in quicksand the shuffled offensive line is a mess it can t pass block or open holes the running game is crippling bad with rbs who miss holes rarely break tackles or try to bounce everything outside and jordan love has been an inaccurate disaster whether the pressure has gotten to the qb who entered his fourth year as a starter or he s simply panicking love s play has been dismal through three games love was pressured 23 times 41 8 pressure rate in</t>
+          <t xml:space="preserve">midway through the third quarter cooper fell to the ground shortly after the snap without being touched and reached for the back of his lower left leg he was visibly distraught on the field and later carted off 34 i 39 m sick 34 quarterback jordan love said 34 he 39 s such an impact player on our defense 34 if cooper 39 s injury ends his season it will be the third such hit to green bay 39 s starting lineup this season right tackle zach bako bewele torn patellar tendon</t>
         </is>
       </c>
       <c r="R138" t="inlineStr">
@@ -10669,7 +10669,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t xml:space="preserve">defensive end a href http www espn com college sports football recruiting player id 259636 zion elee zion elee a the no 2 player in the class in 2025 in state quarterback a href http www espn com college sports football recruiting player id 254623 malik washington malik washington a was one of seven four star sc next 300 signees and immediately won the starting job p p maryland s top graded recruit in 2027 sc next 300 four star wide receiver myles mcafee comes from the same archbishop spalding high school</t>
+          <t xml:space="preserve">maryland 2 3 at no 5 ohio state 4 1 oct 10 at 4 15 p m edt opening line ohio state by 34 5 against the spread ohio state 4 1 maryland 2 3 how to watch btn em key stats em ohio state offense overall 514 4 yards per game 7th in fbs passing 357 yards per game 2nd rushing 157 4 yards per game 71st scoring 42 2 points per game 14th ohio state defense overall 267 yards per game 18th in fbs passing 168 yards per game 24th rushing 99 yards per game 25th scoring 12 6 points per game 8th maryland offense overall 424 yards per game 48th in fbs passing 277 2 yards per game 30th rushing 146 8 yards per game 88th scoring 30 4 points per game 69th maryland defense overall 335 yards per game 56th in fbs pas</t>
         </is>
       </c>
       <c r="R152" t="inlineStr">
@@ -12104,7 +12104,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Bengals WR Ja'Marr Chase suffers concussion in loss to Jaguars | Bengals wide receiver Ja'Marr Chase has been ruled out against the Jaguars with a concussion.</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -12174,7 +12174,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sources: Rams don't intend to limit Puka Nacua's workload | The Rams do not intend to limit Puka Nacua's workload Sunday against the Eagles, sources told ESPN. | sources rams don t intend to limit puka nacua s workload the rams do not intend to limit puka nacua s workload sunday against the eagles sources told espn | Aaron Donald out, Puka Nacua to play in Rams' game vs. | Rams defensive tackle Aaron Donald will not play against the Eagles as he deals with back soreness, while wide receiver Puka Nacua will return from a hip injury after missing the past two games. | aaron donald out puka nacua to play in rams game vs eagles rams defensive tackle aaron donald will not play against the eagles </t>
+          <t xml:space="preserve">n count if there were offseason trophies to hand out los angeles would likely be first in line still for as loaded as this roster is it s imperative the rams stiff arm distractions and keep their heads from getting too high into the clouds puka nacua has a looming potentially top of the market extension and he needs to continue working on himself after a stint in rehab l a already caused a stir when it shocked the nfl world by drafting quarterback ty simpson with the 13th overall pick</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -12524,7 +12524,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t xml:space="preserve">p with 28 seconds left in the fourth quarter sunday afternoon a data clubhouse guid 38248455 3da4 84e4 8090 98b5cc38ffdc href https www espn com nfl team name bal baltimore ravens baltimore ravens a cornerback a data player guid 0fa246a4 1068 3be1 9d79 42844aeedbce href https www espn com nfl player id 4601278 nate wiggins nate wiggins a batted away a pass from a data clubhouse guid b0fc8fb7 9dbe e574 9008 6f0ee7c6b234 href https www espn com nfl team name dal dallas cowboys dallas cowboys a wide receiver a data player guid 2994891b 8927 33cb 6999 e809560d0545 href https www espn com nfl player id 4241389 ceedee lamb ceedee lamb a near the goal line making what many thought was a clutch defe</t>
+          <t xml:space="preserve">CeeDee Lamb's 17 catches, go-ahead score power Cowboys | CeeDee Lamb returned to Houston and caught 17 passes for 189 yards, including the game-winning, 12-yard touchdown with 40 seconds to go, as a large number of family members watched from the stands. | ceedee lamb s 17 catches go ahead score power cowboys ceedee lamb returned to houston and caught 17 passes for 189 yards including the game winning 12 yard touchdown with 40 seconds to go as a large number of family members watched from the stands | Can CeeDee Lamb finish as the overall WR1 in fantasy this season? | can ceedee lamb finish as the overall wr1 in fantasy this season can ceedee lamb finish as the overall wr1 in fantasy this se</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -12804,7 +12804,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vikings WR Justin Jefferson (ankle) out Sunday against Dolphins | Justin Jefferson (ankle) has been ruled out of the team&amp;#x27;s upcoming game against the Dolphins, head coach Kevin O&amp;#x27;Connell said Friday. | vikings wr justin jefferson ankle out sunday against dolphins the minnesota vikings will be without their two time all pro wide receiver on sunday justin jefferson ankle has been ruled out of the team x27 s upcoming game against the dolphins head coach kevin o x27 connell said friday | Vikings' Justin Jefferson out vs. | Vikings WR Justin Jefferson won't play against the Dolphins because of a sprained left ankle, but coach Kevin O'Connell is hopeful he can return in Week 5 vs. | viki</t>
+          <t xml:space="preserve">Vikings WR Justin Jefferson (ankle) out Sunday against Dolphins | Justin Jefferson (ankle) has been ruled out of the team&amp;#x27;s upcoming game against the Dolphins, head coach Kevin O&amp;#x27;Connell said Friday. | vikings wr justin jefferson ankle out sunday against dolphins the minnesota vikings will be without their two time all pro wide receiver on sunday justin jefferson ankle has been ruled out of the team x27 s upcoming game against the dolphins head coach kevin o x27 connell said friday</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -13224,7 +13224,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t xml:space="preserve">very big down for us in these first two games and today we were not good enough and i wasn 39 t good enough fourth down i wasn 39 t good enough as well 34 the first half included encouraging signs for the running game saquon barkley returned from last week 39 s stinger and rushed for 73 yards before halftime his second most in the first half since the start of last season but he finished with 82 yards that shows you how the second half went 34 we know the</t>
+          <t xml:space="preserve">Eagles RB Saquon Barkley leaves loss with hamstring injury | Eagles running back Saquon Barkley has been ruled out of Sunday's game against the Rams with a hamstring injury. | eagles rb saquon barkley leaves loss with hamstring injury eagles running back saquon barkley has been ruled out of sunday s game against the rams with a hamstring injury</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -13854,7 +13854,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">— Carolina Panthers coach Dave Canales was a little worried after Bryce Young and Tetairoa McMillan had some issues connecting on passes in practice. | young mcmillan connect for 2 tds to lead panthers past lions 32 26 carolina panthers coach dave canales was a little worried after bryce young and tetairoa mcmillan had some issues connecting on passes in practice</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -14064,7 +14064,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who unseats Josh Allen at the top of Nick Shook&amp;#x27;s QB rankings? | nfl and the longest of herbert s career the chargers failed to capitalize on five forced turnovers on sunday as the offense struggled to punch in scores going 1 of 4 in the red zone as the defense gave l a repeated chances to thwart josh allen s bills herbert and co never found a groove after three weeks it s been a rusty operation and herbert doesn t appear comfortable in the scheme yet the interior of the offensive line getting repeatedly blasted doesn t help also the pass catching corps</t>
+          <t xml:space="preserve">is still turning the ball over at a discomforting rate the running game remains an issue the pass rush hasn 39 t been anything special but with their quarterback finally playing like the guy who can carry a team and with their defense slowing down josh allen and the bills like no other unit had everything is on the table for the patriots of course a lot of that is because of maye the disasters of his first three weeks were pretty much gone with allen on the opposing sideline maye certainly</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t xml:space="preserve">NFL news roundup: Lamar Jackson (back) limited at practice; | nfl news roundup lamar jackson back limited at practice falcons extend dt gervon dexter nfl com keeps you up to date with all of the latest league news from around the nfl visit nfl com x27 s transaction hub for a daily breakdown</t>
+          <t xml:space="preserve">Ravens quarterback Lamar Jackson exits win over Titans early due to ankle injury | Baltimore Ravens quarterback Lamar Jackson suffered an ankle injury in the first half of Sunday&amp;#x27;s 24-18 win over the Tennessee Titans and did not return. | baltimore ravens quarterback lamar jackson suffered an ankle injury in the first half of sunday s 24 18 win over the tennessee titans and did not return jackson appeared to suffer the injury when he was sacked on one of the final plays of the first half lamar s dealing with a little bit of an ankle head coach jesse minter told reporters after the game don t know enough about it right now we ll have to see where that s at nfl network insider ian rapopor</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -14694,7 +14694,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t xml:space="preserve">jacksonville fla jacksonville jaguars cornerback travis hunter ended up with the football from his first nfl interception hunter spun the ball in celebration and then danced in the end zone after picking off a pass from new england patriots quarterback drake maye late in the second quarter sunday a patriots ball boy picked it up and refused to give it to jaguars veteran defensive end josh hines allen even screaming hey you can t touch me when hines allen tried to grab the ball the ball boy appeared to try to push hines allen away nfl players are allowed to keep game balls although they get charged a hefty price by the league hines allen tried to knock this one out of the ball boy s hands bef</t>
+          <t xml:space="preserve">Drake Maye rebounds as Patriots hand Bills first defeat | Drake Maye snapped out of his early-season slide with a clutch performance as the New England Patriots upset the Buffalo Bills 29-26 at Highmark Stadium in a result that coach Mike Vrabel highlighted as critical for the defending AFC champions. | drake maye rebounds as patriots hand bills first defeat drake maye snapped out of his early season slide with a clutch performance as the new england patriots upset the buffalo bills 29 26 at highmark stadium in a result that coach mike vrabel highlighted as critical for the defending afc champions | Why Adam Rank is still rolling with Drake Maye as a fantasy starter for now | why adam rank i</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Michael Florio: Fantasy managers shouldn't think twice about starting Javonte Williams | michael florio fantasy managers shouldn t think twice about starting javonte williams michael florio fantasy managers shouldn t think twice about starting javonte williams</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
@@ -16304,7 +16304,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sources: Sam LaPorta, Lions break off contract talks | The Lions and star tight end Sam LaPorta have broken off contract talks, sources told NFL Network, after attempting to work out a long-term deal for the first few weeks of the season. | sources sam laporta lions break off contract talks the lions and star tight end sam laporta have broken off contract talks sources told nfl network after attempting to work out a long term deal for the first few weeks of the season | en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of </t>
+          <t xml:space="preserve">en in front of extensions in recent years so everyone expects a top of the rb market contract for gibbs to come barreling down the pike 3 can detroit return to health detroit has significant injuries to track at the onset of camp tight end sam laporta is the name to watch on offense but the defense has greater concerns brian branch suffered a late season achilles tear and while the lions haven t put a hard timeline on the safety s recovery it will be a surprise if he s good to go to ope</t>
         </is>
       </c>
       <c r="R64" t="inlineStr">
@@ -16514,7 +16514,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Will Marcus Mariota lead Washington to a second straight win in relief of Jayden Daniels? | cam bynum boasts an impressive track record in international games heading into sunday s matchup with the commanders at london s tottenham hotspur stadium the colts safety has made three previous international appearances two in london with the vikings and another in germany last year for indianapolis and has come away 3 0 with 17 tackles two passes defensed an interception and a forced fumble what has contributed to such a boost overseas for the 28 year old he believes a lot of it boils down to the atmosphere whenever i m having fun and feeling loose that s when i play the best football bynum told mi</t>
+          <t xml:space="preserve">ruled out at halftime mariota was playing in place of washington starter jayden daniels who has been sidelined the last two weeks after dislocating his left elbow on sept 20 commanders coach dan quinn said after the loss that mariota is feared to have aggravated an mcl injury that sidelined him in 2022 the vet qb will undergo testing to confirm the nature of the injury mariota suffered the knee injury on a third down sack midway through the first quarter when indy defensive end laiatu latu landed on the veteran qb s right leg mariota went to the locker room and was replaced by kaliakmanis with washington leading 6 0 this was kaliakmanis first nfl regular season game appearance the 23 year ol</t>
         </is>
       </c>
       <c r="R67" t="inlineStr">
@@ -18194,7 +18194,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Placed WR Jayden Reed on injured reserve. | transaction signed g kevin zeitler placed wr jayden reed on injured reserve signed dt david blay and wr coleman owen to the practice squad signed g kevin zeitler placed wr jayden reed on injured reserve signed dt david blay and wr coleman owen to the practice squad | Placed WR Jayden Reed on injured reserve.</t>
+          <t xml:space="preserve">39 s such an impact player on our defense 34 if cooper 39 s injury ends his season it will be the third such hit to green bay 39 s starting lineup this season right tackle zach bako bewele torn patellar tendon and wide receiver jayden reed neck are both out for the year too the packers will now rely on special teams captain and linebacker isaiah mcduffie to fill cooper 39 s spot in the starting lineup alongside veteran zaire franklin lafleur was visibly frustrated during his postgame press conference likely | Placed WR Jayden Reed on injured reserve. | transaction signed g kevin zeitler placed wr jayden reed on injured reserve signed dt david blay and wr coleman owen to the practice squad si</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -18264,7 +18264,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Seahawks place RB Jadarian Price (chest) on injured reserve | Running back Jadarian Price&amp;#x27;s slow start to his rookie season just hit another snag. | seahawks place rb jadarian price chest on injured reserve running back jadarian price x27 s slow start to his rookie season just hit another snag the seahawks are placing price on injured reserve due to a chest injury espn x27 s adam schefter reported saturday | Seahawks place RB Jadarian Price (chest) on IR | The Seattle Seahawks are placing starting running back Jadarian Price on injured reserve, the team announced Saturday. | seahawks place rb jadarian price chest on ir the seattle seahawks are placing starting running back jadarian pric</t>
+          <t xml:space="preserve">Seahawks place RB Jadarian Price (chest) on injured reserve | Running back Jadarian Price&amp;#x27;s slow start to his rookie season just hit another snag. | seahawks place rb jadarian price chest on injured reserve running back jadarian price x27 s slow start to his rookie season just hit another snag the seahawks are placing price on injured reserve due to a chest injury espn x27 s adam schefter reported saturday</t>
         </is>
       </c>
       <c r="R92" t="inlineStr">
@@ -21064,7 +21064,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t xml:space="preserve">defensive end a href http www espn com college sports football recruiting player id 259636 zion elee zion elee a the no 2 player in the class in 2025 in state quarterback a href http www espn com college sports football recruiting player id 254623 malik washington malik washington a was one of seven four star sc next 300 signees and immediately won the starting job p p maryland s top graded recruit in 2027 sc next 300 four star wide receiver myles mcafee comes from the same archbishop spalding high school</t>
+          <t xml:space="preserve">maryland 2 3 at no 5 ohio state 4 1 oct 10 at 4 15 p m edt opening line ohio state by 34 5 against the spread ohio state 4 1 maryland 2 3 how to watch btn em key stats em ohio state offense overall 514 4 yards per game 7th in fbs passing 357 yards per game 2nd rushing 157 4 yards per game 71st scoring 42 2 points per game 14th ohio state defense overall 267 yards per game 18th in fbs passing 168 yards per game 24th rushing 99 yards per game 25th scoring 12 6 points per game 8th maryland offense overall 424 yards per game 48th in fbs passing 277 2 yards per game 30th rushing 146 8 yards per game 88th scoring 30 4 points per game 69th maryland defense overall 335 yards per game 56th in fbs pas</t>
         </is>
       </c>
       <c r="R132" t="inlineStr">
@@ -22534,7 +22534,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t xml:space="preserve">— The Carolina Panthers found themselves in a precarious position last November, facing a red hot Matthew Stafford without three defensive starters, including standout cornerback Jaycee Horn.</t>
+          <t xml:space="preserve">Matthew Stafford says Nacua 'played like Puka' in return for Rams</t>
         </is>
       </c>
       <c r="R153" t="inlineStr">
@@ -22814,7 +22814,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sources: Baker Mayfield return hinges on when QB can grip football | Baker Mayfield is expected to miss anywhere from three to six weeks, sources told ESPN, depending on how quickly the Bucs QB can grip the football. | p a data clubhouse guid 13e8b157 a75a ff24 ae91 fa3d52ddf204 href https www espn com nfl team name tb tampa bay buccaneers tampa bay buccaneers a head coach todd bowles says a data player guid 5bb4376a d089 e3e4 e49a 44f1d709a012 href https www espn com nfl player id 3052587 baker mayfield baker mayfield a will miss at least three weeks due to his dislocated right thumb but that is the minimum p p there is a flipside scenario as well p p sources told espn that mayfield is deal</t>
+          <t xml:space="preserve">Sources: Baker Mayfield return hinges on when QB can grip football | Baker Mayfield is expected to miss anywhere from three to six weeks, sources told ESPN, depending on how quickly the Buccaneers quarterback can grip the football. | sources baker mayfield return hinges on when qb can grip football baker mayfield is expected to miss anywhere from three to six weeks sources told espn depending on how quickly the buccaneers quarterback can grip the football</t>
         </is>
       </c>
       <c r="R157" t="inlineStr">
@@ -22954,7 +22954,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t xml:space="preserve">an offense playing as if it s in quicksand the shuffled offensive line is a mess it can t pass block or open holes the running game is crippling bad with rbs who miss holes rarely break tackles or try to bounce everything outside and jordan love has been an inaccurate disaster whether the pressure has gotten to the qb who entered his fourth year as a starter or he s simply panicking love s play has been dismal through three games love was pressured 23 times 41 8 pressure rate in</t>
+          <t xml:space="preserve">midway through the third quarter cooper fell to the ground shortly after the snap without being touched and reached for the back of his lower left leg he was visibly distraught on the field and later carted off 34 i 39 m sick 34 quarterback jordan love said 34 he 39 s such an impact player on our defense 34 if cooper 39 s injury ends his season it will be the third such hit to green bay 39 s starting lineup this season right tackle zach bako bewele torn patellar tendon</t>
         </is>
       </c>
       <c r="R159" t="inlineStr">

</xml_diff>

<commit_message>
Withhold weekly model scores alongside unavailable current ranks
</commit_message>
<xml_diff>
--- a/exports/fantasy-2026-current.xlsx
+++ b/exports/fantasy-2026-current.xlsx
@@ -13971,17 +13971,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Patrick Mahomes II</t>
+          <t xml:space="preserve">CeeDee Lamb</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kansas City Chiefs</t>
+          <t xml:space="preserve">Dallas Cowboys</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D2">
@@ -13997,8 +13997,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G2">
-        <v>9.29568</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -14006,33 +14008,33 @@
         </is>
       </c>
       <c r="I2">
-        <v>84</v>
+        <v>9</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">QB13</t>
+          <t xml:space="preserve">WR5</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">CeeDee Lamb</t>
+          <t xml:space="preserve">Kenneth Walker III</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dallas Cowboys</t>
+          <t xml:space="preserve">Kansas City Chiefs</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">RB</t>
         </is>
       </c>
       <c r="D3">
@@ -14048,8 +14050,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G3">
-        <v>8.91456</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -14057,28 +14061,28 @@
         </is>
       </c>
       <c r="I3">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR5</t>
+          <t xml:space="preserve">RB11</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rashee Rice</t>
+          <t xml:space="preserve">A.J. Brown</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kansas City Chiefs</t>
+          <t xml:space="preserve">New England Patriots</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -14099,37 +14103,39 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G4">
-        <v>8.74848</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNKNOWN</t>
+          <t xml:space="preserve">EXPECTED_INACTIVE</t>
         </is>
       </c>
       <c r="I4">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR18</t>
+          <t xml:space="preserve">WR10</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">George Pickens</t>
+          <t xml:space="preserve">Tetairoa McMillan</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dallas Cowboys</t>
+          <t xml:space="preserve">Carolina Panthers</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -14150,8 +14156,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G5">
-        <v>8.66688</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -14159,33 +14167,33 @@
         </is>
       </c>
       <c r="I5">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR13</t>
+          <t xml:space="preserve">WR12</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kenneth Walker III</t>
+          <t xml:space="preserve">George Pickens</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kansas City Chiefs</t>
+          <t xml:space="preserve">Dallas Cowboys</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D6">
@@ -14201,8 +14209,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G6">
-        <v>8.6592</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -14210,33 +14220,33 @@
         </is>
       </c>
       <c r="I6">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB11</t>
+          <t xml:space="preserve">WR13</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dak Prescott</t>
+          <t xml:space="preserve">Rashee Rice</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dallas Cowboys</t>
+          <t xml:space="preserve">Kansas City Chiefs</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">QB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D7">
@@ -14252,8 +14262,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G7">
-        <v>8.65152</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -14261,23 +14273,23 @@
         </is>
       </c>
       <c r="I7">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">QB15</t>
+          <t xml:space="preserve">WR18</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jalon Daniels</t>
+          <t xml:space="preserve">Emeka Egbuka</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -14287,7 +14299,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">QB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D8">
@@ -14303,8 +14315,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G8">
-        <v>8.63146</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -14312,11 +14326,11 @@
         </is>
       </c>
       <c r="I8">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">QB6</t>
+          <t xml:space="preserve">WR19</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -14328,17 +14342,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tetairoa McMillan</t>
+          <t xml:space="preserve">Javonte Williams</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carolina Panthers</t>
+          <t xml:space="preserve">Dallas Cowboys</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">RB</t>
         </is>
       </c>
       <c r="D9">
@@ -14354,8 +14368,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G9">
-        <v>8.63136</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -14363,23 +14379,23 @@
         </is>
       </c>
       <c r="I9">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR12</t>
+          <t xml:space="preserve">RB15</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Baker Mayfield</t>
+          <t xml:space="preserve">Bucky Irving</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -14389,7 +14405,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">QB</t>
+          <t xml:space="preserve">RB</t>
         </is>
       </c>
       <c r="D10">
@@ -14405,8 +14421,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G10">
-        <v>8.56896</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -14414,11 +14432,11 @@
         </is>
       </c>
       <c r="I10">
-        <v>186</v>
+        <v>48</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">QB25</t>
+          <t xml:space="preserve">RB16</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -14430,7 +14448,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ted Hurst III</t>
+          <t xml:space="preserve">Jalon Daniels</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -14440,7 +14458,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">QB</t>
         </is>
       </c>
       <c r="D11">
@@ -14456,20 +14474,22 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G11">
-        <v>8.325</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXPECTED_ACTIVE</t>
+          <t xml:space="preserve">UNKNOWN</t>
         </is>
       </c>
       <c r="I11">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR35</t>
+          <t xml:space="preserve">QB6</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -14481,17 +14501,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Javonte Williams</t>
+          <t xml:space="preserve">Marvin Harrison Jr.</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dallas Cowboys</t>
+          <t xml:space="preserve">Arizona Cardinals</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D12">
@@ -14507,32 +14527,34 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G12">
-        <v>8.25696</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNKNOWN</t>
+          <t xml:space="preserve">EXPECTED_INACTIVE</t>
         </is>
       </c>
       <c r="I12">
-        <v>47</v>
+        <v>74</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB15</t>
+          <t xml:space="preserve">WR34</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emeka Egbuka</t>
+          <t xml:space="preserve">Ted Hurst III</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -14558,20 +14580,22 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G13">
-        <v>8.19264</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNKNOWN</t>
+          <t xml:space="preserve">EXPECTED_ACTIVE</t>
         </is>
       </c>
       <c r="I13">
-        <v>36</v>
+        <v>75</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR19</t>
+          <t xml:space="preserve">WR35</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -14583,17 +14607,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bucky Irving</t>
+          <t xml:space="preserve">Patrick Mahomes II</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tampa Bay Buccaneers</t>
+          <t xml:space="preserve">Kansas City Chiefs</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB</t>
+          <t xml:space="preserve">QB</t>
         </is>
       </c>
       <c r="D14">
@@ -14609,8 +14633,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G14">
-        <v>8.0064</v>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -14618,33 +14644,33 @@
         </is>
       </c>
       <c r="I14">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB16</t>
+          <t xml:space="preserve">QB13</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Travis Kelce</t>
+          <t xml:space="preserve">Dak Prescott</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kansas City Chiefs</t>
+          <t xml:space="preserve">Dallas Cowboys</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">TE</t>
+          <t xml:space="preserve">QB</t>
         </is>
       </c>
       <c r="D15">
@@ -14660,8 +14686,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G15">
-        <v>7.944</v>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -14669,28 +14697,28 @@
         </is>
       </c>
       <c r="I15">
-        <v>132</v>
+        <v>103</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t xml:space="preserve">TE21</t>
+          <t xml:space="preserve">QB15</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jake Ferguson</t>
+          <t xml:space="preserve">Darren Waller</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dallas Cowboys</t>
+          <t xml:space="preserve">Carolina Panthers</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -14711,8 +14739,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G16">
-        <v>7.87104</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -14720,28 +14750,28 @@
         </is>
       </c>
       <c r="I16">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t xml:space="preserve">TE15</t>
+          <t xml:space="preserve">TE14</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Darren Waller</t>
+          <t xml:space="preserve">Jake Ferguson</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carolina Panthers</t>
+          <t xml:space="preserve">Dallas Cowboys</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -14762,8 +14792,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G17">
-        <v>7.79362</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -14771,33 +14803,33 @@
         </is>
       </c>
       <c r="I17">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t xml:space="preserve">TE14</t>
+          <t xml:space="preserve">TE15</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chuba Hubbard</t>
+          <t xml:space="preserve">Mack Hollins</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carolina Panthers</t>
+          <t xml:space="preserve">New England Patriots</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D18">
@@ -14813,42 +14845,44 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G18">
-        <v>7.7328</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNKNOWN</t>
+          <t xml:space="preserve">EXPECTED_INACTIVE</t>
         </is>
       </c>
       <c r="I18">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB41</t>
+          <t xml:space="preserve">WR55</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chris Godwin Jr.</t>
+          <t xml:space="preserve">Travis Kelce</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tampa Bay Buccaneers</t>
+          <t xml:space="preserve">Kansas City Chiefs</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">TE</t>
         </is>
       </c>
       <c r="D19">
@@ -14864,8 +14898,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G19">
-        <v>7.54176</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -14873,28 +14909,28 @@
         </is>
       </c>
       <c r="I19">
-        <v>151</v>
+        <v>132</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR65</t>
+          <t xml:space="preserve">TE21</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jalen Coker</t>
+          <t xml:space="preserve">Xavier Worthy</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Carolina Panthers</t>
+          <t xml:space="preserve">Kansas City Chiefs</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -14915,8 +14951,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G20">
-        <v>7.47936</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -14924,11 +14962,11 @@
         </is>
       </c>
       <c r="I20">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR61</t>
+          <t xml:space="preserve">WR59</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -14940,17 +14978,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Xavier Worthy</t>
+          <t xml:space="preserve">Kenneth Gainwell</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kansas City Chiefs</t>
+          <t xml:space="preserve">Tampa Bay Buccaneers</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">RB</t>
         </is>
       </c>
       <c r="D21">
@@ -14966,8 +15004,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G21">
-        <v>7.1856</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -14975,23 +15015,23 @@
         </is>
       </c>
       <c r="I21">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR59</t>
+          <t xml:space="preserve">RB38</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jonathon Brooks</t>
+          <t xml:space="preserve">Jalen Coker</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -15001,7 +15041,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D22">
@@ -15017,8 +15057,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G22">
-        <v>7.18176</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -15026,11 +15068,11 @@
         </is>
       </c>
       <c r="I22">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB45</t>
+          <t xml:space="preserve">WR61</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -15042,12 +15084,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kenneth Gainwell</t>
+          <t xml:space="preserve">Chuba Hubbard</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tampa Bay Buccaneers</t>
+          <t xml:space="preserve">Carolina Panthers</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -15068,8 +15110,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G23">
-        <v>7.15776</v>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -15077,33 +15121,33 @@
         </is>
       </c>
       <c r="I23">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB38</t>
+          <t xml:space="preserve">RB41</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emmett Johnson</t>
+          <t xml:space="preserve">Michael Pittman Jr.</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kansas City Chiefs</t>
+          <t xml:space="preserve">Pittsburgh Steelers</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D24">
@@ -15119,42 +15163,44 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G24">
-        <v>7.15536</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t xml:space="preserve">UNKNOWN</t>
+          <t xml:space="preserve">EXPECTED_INACTIVE</t>
         </is>
       </c>
       <c r="I24">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB43</t>
+          <t xml:space="preserve">WR62</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
+          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">A.J. Brown</t>
+          <t xml:space="preserve">Emmett Johnson</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">New England Patriots</t>
+          <t xml:space="preserve">Kansas City Chiefs</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">RB</t>
         </is>
       </c>
       <c r="D25">
@@ -15170,42 +15216,44 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G25">
-        <v>6.85894</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXPECTED_INACTIVE</t>
+          <t xml:space="preserve">UNKNOWN</t>
         </is>
       </c>
       <c r="I25">
-        <v>25</v>
+        <v>143</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR10</t>
+          <t xml:space="preserve">RB43</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marvin Harrison Jr.</t>
+          <t xml:space="preserve">Jonathon Brooks</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Arizona Cardinals</t>
+          <t xml:space="preserve">Carolina Panthers</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">RB</t>
         </is>
       </c>
       <c r="D26">
@@ -15221,37 +15269,39 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G26">
-        <v>6.2085</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXPECTED_INACTIVE</t>
+          <t xml:space="preserve">UNKNOWN</t>
         </is>
       </c>
       <c r="I26">
-        <v>74</v>
+        <v>147</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR34</t>
+          <t xml:space="preserve">RB45</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
+          <t xml:space="preserve">NO_CURRENT_WEEK_GAME</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Michael Pittman Jr.</t>
+          <t xml:space="preserve">Chris Godwin Jr.</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pittsburgh Steelers</t>
+          <t xml:space="preserve">Tampa Bay Buccaneers</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -15272,42 +15322,44 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G27">
-        <v>5.9925</v>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXPECTED_INACTIVE</t>
+          <t xml:space="preserve">UNKNOWN</t>
         </is>
       </c>
       <c r="I27">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR62</t>
+          <t xml:space="preserve">WR65</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
+          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mack Hollins</t>
+          <t xml:space="preserve">Jonah Coleman</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">New England Patriots</t>
+          <t xml:space="preserve">Denver Broncos</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">RB</t>
         </is>
       </c>
       <c r="D28">
@@ -15323,8 +15375,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G28">
-        <v>5.84321</v>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -15332,11 +15386,11 @@
         </is>
       </c>
       <c r="I28">
-        <v>126</v>
+        <v>154</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR55</t>
+          <t xml:space="preserve">RB48</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -15348,12 +15402,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jonah Coleman</t>
+          <t xml:space="preserve">Tank Bigsby</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Denver Broncos</t>
+          <t xml:space="preserve">Philadelphia Eagles</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -15374,8 +15428,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G29">
-        <v>5.31</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -15383,11 +15439,11 @@
         </is>
       </c>
       <c r="I29">
-        <v>154</v>
+        <v>181</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB48</t>
+          <t xml:space="preserve">RB62</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -15399,17 +15455,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tank Dell</t>
+          <t xml:space="preserve">Baker Mayfield</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Houston Texans</t>
+          <t xml:space="preserve">Tampa Bay Buccaneers</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR</t>
+          <t xml:space="preserve">QB</t>
         </is>
       </c>
       <c r="D30">
@@ -15425,42 +15481,44 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G30">
-        <v>5.0025</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t xml:space="preserve">EXPECTED_INACTIVE</t>
+          <t xml:space="preserve">UNKNOWN</t>
         </is>
       </c>
       <c r="I30">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t xml:space="preserve">WR74</t>
+          <t xml:space="preserve">QB25</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
+          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tank Bigsby</t>
+          <t xml:space="preserve">Tank Dell</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Philadelphia Eagles</t>
+          <t xml:space="preserve">Houston Texans</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB</t>
+          <t xml:space="preserve">WR</t>
         </is>
       </c>
       <c r="D31">
@@ -15476,8 +15534,10 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="G31">
-        <v>4.94625</v>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -15485,11 +15545,11 @@
         </is>
       </c>
       <c r="I31">
-        <v>181</v>
+        <v>195</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t xml:space="preserve">RB62</t>
+          <t xml:space="preserve">WR74</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">

</xml_diff>

<commit_message>
Run ordered weekly production lifecycle
</commit_message>
<xml_diff>
--- a/exports/fantasy-2026-current.xlsx
+++ b/exports/fantasy-2026-current.xlsx
@@ -17035,7 +17035,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_ADVERSE_STATUS_REPORTED</t>
+          <t xml:space="preserve">QUESTIONABLE</t>
         </is>
       </c>
       <c r="I61">
@@ -21116,7 +21116,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t xml:space="preserve">NO_ADVERSE_STATUS_REPORTED</t>
+          <t xml:space="preserve">OUT</t>
         </is>
       </c>
       <c r="I138">
@@ -21129,7 +21129,7 @@
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAME_STARTED_NO_ORIGINAL_WEEKLY_RANK</t>
+          <t xml:space="preserve">NOT_EXPECTED_TO_PLAY</t>
         </is>
       </c>
     </row>

</xml_diff>